<commit_message>
Ajoute un dossier prêt pour Netlify Drop (non indexé)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KdRfZ77NaKjBozcXZxFJio
</commit_message>
<xml_diff>
--- a/dist/Tableau_de_bord_Mali.xlsx
+++ b/dist/Tableau_de_bord_Mali.xlsx
@@ -15168,12 +15168,12 @@
       </c>
       <c r="L4" s="61" t="inlineStr">
         <is>
+          <t>Civils</t>
+        </is>
+      </c>
+      <c r="M4" s="61" t="inlineStr">
+        <is>
           <t>Groupes armés</t>
-        </is>
-      </c>
-      <c r="M4" s="61" t="inlineStr">
-        <is>
-          <t>Civils</t>
         </is>
       </c>
       <c r="N4" s="61" t="inlineStr">
@@ -15465,7 +15465,7 @@
     <row r="10">
       <c r="B10" s="42" t="inlineStr">
         <is>
-          <t>Attaque ciblée / VIP</t>
+          <t>Affrontement JNIM–EIS</t>
         </is>
       </c>
       <c r="C10" s="47">
@@ -15575,7 +15575,7 @@
     <row r="12">
       <c r="B12" s="42" t="inlineStr">
         <is>
-          <t>Affrontement JNIM–EIS</t>
+          <t>Attaque ciblée / VIP</t>
         </is>
       </c>
       <c r="C12" s="47">
@@ -15740,7 +15740,7 @@
     <row r="15">
       <c r="B15" s="42" t="inlineStr">
         <is>
-          <t>Tirs indirects</t>
+          <t>Lutte anti-drone</t>
         </is>
       </c>
       <c r="C15" s="47">
@@ -15795,7 +15795,7 @@
     <row r="16">
       <c r="B16" s="42" t="inlineStr">
         <is>
-          <t>Lutte anti-drone</t>
+          <t>Tirs indirects</t>
         </is>
       </c>
       <c r="C16" s="47">

</xml_diff>